<commit_message>
Remove outdated operation report and update associated Excel file
</commit_message>
<xml_diff>
--- a/修正内容報告_20260817-18.xlsx
+++ b/修正内容報告_20260817-18.xlsx
@@ -567,7 +567,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>・完了工事一覧に「計画」タブを追加し、通常画面と同じ3タブ構成に変更</t>
+          <t>完了工事一覧に「計画」タブを追加し、通常画面と同じ3タブ構成に変更</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>・表の列見出しにフィルター・並べ替え機能を追加（従来の絞り込みボタンは廃止）</t>
+          <t>表の列見出しにフィルター・並べ替え機能を追加（従来の絞り込みボタンは廃止）</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>・担当別画面でバーをドラッグして移動・伸縮できるように改善</t>
+          <t>担当別画面でバーをドラッグして移動・伸縮できるように改善</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>・表の列幅をドラッグで自由に調整できるように改善</t>
+          <t>表の列幅をドラッグで自由に調整できるように改善</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>・ガントバー・担当別バーの表示に工事番号・機械名を追加</t>
+          <t>ガントバー・担当別バーの表示に工事番号・機械名を追加</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>・担当者プルダウンに「未定」を追加</t>
+          <t>担当者プルダウンに「未定」を追加</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>・担当別画面の並び順を開始日順に変更し、機械名も表示</t>
+          <t>担当別画面の並び順を開始日順に変更し、機械名も表示</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>・タスク編集画面（ライトボックス）を拡大して見やすく改善</t>
+          <t>タスク編集画面（ライトボックス）を拡大して見やすく改善</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>・画面上部のボタン配置を整理</t>
+          <t>画面上部のボタン配置を整理</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>・開始日・終了日を個別編集すると他方まで変わってしまう不具合を修正</t>
+          <t>開始日・終了日を個別編集すると他方まで変わってしまう不具合を修正</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>・担当別フルスクリーン表示の崩れを修正</t>
+          <t>担当別フルスクリーン表示の崩れを修正</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>・担当別フルスクリーンでダブルクリック編集ができない不具合を修正</t>
+          <t>担当別フルスクリーンでダブルクリック編集ができない不具合を修正</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>・工事番号未選択でも新規タスクを追加できるよう修正</t>
+          <t>工事番号未選択でも新規タスクを追加できるよう修正</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>・「現地試運転」モードを廃止し「出張」モードに統合</t>
+          <t>「現地試運転」モードを廃止し「出張」モードに統合</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>・表示モードボタンの再クリックで担当別画面に戻らない仕様に変更</t>
+          <t>表示モードボタンの再クリックで担当別画面に戻らない仕様に変更</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>・「試運転」の表記を「社内試運転」に統一</t>
+          <t>「試運転」の表記を「社内試運転」に統一</t>
         </is>
       </c>
     </row>

</xml_diff>